<commit_message>
fix(export): preserve canonical XLSX behavior [B]
</commit_message>
<xml_diff>
--- a/docs/program/EXPORT_1_XLSX_20260916/artifacts/northwind-supplier-scorecard.xlsx
+++ b/docs/program/EXPORT_1_XLSX_20260916/artifacts/northwind-supplier-scorecard.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Data" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Supplier scorecard" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Summary" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Data'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Supplier scorecard'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -158,40 +158,40 @@
       <b/>
       <color rgb="FF1B2A41"/>
       <sz val="16"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <color rgb="FF46556B"/>
       <sz val="10.5"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <color rgb="FF667085"/>
       <sz val="9"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FF1B2A41"/>
       <sz val="10"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <color rgb="FF101828"/>
       <sz val="10"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
     <font>
       <i/>
       <color rgb="FF667085"/>
       <sz val="9"/>
-      <name val="Aptos"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
@@ -381,7 +381,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFCE8E6"/>
+          <bgColor rgb="FFFCE8E6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -392,7 +392,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE3F5E9"/>
+          <bgColor rgb="FFE3F5E9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1156,7 +1156,7 @@
         <v>32</v>
       </c>
       <c r="B4" s="27">
-        <f>COUNTA('Data'!A7:A11)</f>
+        <f>COUNTA('Supplier scorecard'!A7:A11)</f>
       </c>
       <c r="C4" s="26" t="s">
         <v>33</v>
@@ -1167,7 +1167,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="29">
-        <f>SUM('Data'!C7:C11)</f>
+        <f>SUM('Supplier scorecard'!C7:C11)</f>
       </c>
       <c r="C5" s="28" t="s">
         <v>34</v>
@@ -1178,7 +1178,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="30">
-        <f>SUM('Data'!D7:D11)/SUM('Data'!C7:C11)</f>
+        <f>SUM('Supplier scorecard'!D7:D11)/SUM('Supplier scorecard'!C7:C11)</f>
       </c>
       <c r="C6" s="26" t="s">
         <v>35</v>
@@ -1189,7 +1189,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="29">
-        <f>SUM('Data'!F7:F11)</f>
+        <f>SUM('Supplier scorecard'!F7:F11)</f>
       </c>
       <c r="C7" s="28" t="s">
         <v>36</v>
@@ -1200,7 +1200,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="30">
-        <f>SUM('Data'!G7:G11)/SUM('Data'!F7:F11)</f>
+        <f>SUM('Supplier scorecard'!G7:G11)/SUM('Supplier scorecard'!F7:F11)</f>
       </c>
       <c r="C8" s="26" t="s">
         <v>37</v>
@@ -1211,7 +1211,7 @@
         <v>38</v>
       </c>
       <c r="B9" s="29">
-        <f>COUNTIF('Data'!J7:J11,"Worsening")</f>
+        <f>COUNTIF('Supplier scorecard'!J7:J11,"Worsening")</f>
       </c>
       <c r="C9" s="28" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
fix(export): wire SHEET-BASE XLSX profile [B]
</commit_message>
<xml_diff>
--- a/docs/program/EXPORT_1_XLSX_20260916/artifacts/northwind-supplier-scorecard.xlsx
+++ b/docs/program/EXPORT_1_XLSX_20260916/artifacts/northwind-supplier-scorecard.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Supplier scorecard" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Summary" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Template fields" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Supplier scorecard'!$6:$6</definedName>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="54">
   <si>
     <t>Supplier Quality Scorecard</t>
   </si>
@@ -23,7 +23,7 @@
     <t>Goods-in nonconformances · Q2 to Q3</t>
   </si>
   <si>
-    <t>Northwind Manufacturing Ltd.  ·  Consultify → Materials → Sheets  ·  Generated 2026-09-16  ·  Confidential</t>
+    <t>Northwind Manufacturing Ltd.  ·  Consultify → Materials → Sheets  ·  Generated 2026-09-17  ·  Confidential</t>
   </si>
   <si>
     <t>Supplier</t>
@@ -101,50 +101,91 @@
     <t>Tolerance: NC rate above 3.0% triggers enhanced surveillance. Δ pp above +0.3 marks a worsening supplier. NC rate and Δ are formulas, not pasted values.</t>
   </si>
   <si>
-    <t>Supplier Quality Scorecard — Summary</t>
-  </si>
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Suppliers</t>
-  </si>
-  <si>
-    <t>Data!A</t>
-  </si>
-  <si>
-    <t>Data!C</t>
-  </si>
-  <si>
-    <t>Data!C:D</t>
-  </si>
-  <si>
-    <t>Data!F</t>
-  </si>
-  <si>
-    <t>Data!F:G</t>
-  </si>
-  <si>
-    <t>Worsening suppliers</t>
-  </si>
-  <si>
-    <t>Data!J</t>
+    <t>Cell / range</t>
+  </si>
+  <si>
+    <t>What it is</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Bound to</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>Template field</t>
+  </si>
+  <si>
+    <t>Template</t>
+  </si>
+  <si>
+    <t>Fixed title of the template</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>Generator content</t>
+  </si>
+  <si>
+    <t>Generator</t>
+  </si>
+  <si>
+    <t>Reporting period selected at generation</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>Org name · source path · date · confidentiality label</t>
+  </si>
+  <si>
+    <t>A6:K6</t>
+  </si>
+  <si>
+    <t>Column set, labels, widths, freeze, autofilter</t>
+  </si>
+  <si>
+    <t>A7:D11, F7:G11, K7:K11</t>
+  </si>
+  <si>
+    <t>Supplier register + goods-in nonconformance records</t>
+  </si>
+  <si>
+    <t>E, H, I, J columns</t>
+  </si>
+  <si>
+    <t>Template formula</t>
+  </si>
+  <si>
+    <t>NC rate, Δ pp and trend label — computed, never pasted</t>
+  </si>
+  <si>
+    <t>Row 12</t>
+  </si>
+  <si>
+    <t>SUM + weighted NC rate (not average of averages)</t>
+  </si>
+  <si>
+    <t>Conditional formats</t>
+  </si>
+  <si>
+    <t>Template rule</t>
+  </si>
+  <si>
+    <t>Tolerance 3.0% · Δ ±0.3 pp · trend colours</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="+0.0;-0.0;0.0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.##"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -288,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -352,12 +393,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1097,10 +1141,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7:J12">
-    <cfRule type="containsText" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISERROR(SEARCH("Worsening",J7)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>NOT(ISERROR(SEARCH("Improving",J7)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1125,102 +1169,142 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="B1" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="C1" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="D1" s="25" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="27">
-        <f>COUNTA('Supplier scorecard'!A7:A11)</f>
+        <v>40</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>33</v>
       </c>
       <c r="C4" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="27" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="29">
-        <f>SUM('Supplier scorecard'!C7:C11)</f>
-      </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="27" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="27" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="30">
-        <f>SUM('Supplier scorecard'!D7:D11)/SUM('Supplier scorecard'!C7:C11)</f>
+        <v>44</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>37</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="29">
-        <f>SUM('Supplier scorecard'!F7:F11)</f>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="30">
-        <f>SUM('Supplier scorecard'!G7:G11)/SUM('Supplier scorecard'!F7:F11)</f>
+        <v>49</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>47</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="29">
-        <f>COUNTIF('Supplier scorecard'!J7:J11,"Worsening")</f>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>39</v>
+        <v>34</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9Consultify&amp;R&amp;9Northwind Manufacturing Ltd.</oddHeader>

</xml_diff>